<commit_message>
1.10.2: kode nomor dokumen FDS diganti FI
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H4ZVrZ9V3BgNkxuhZCNDSa
</commit_message>
<xml_diff>
--- a/dokumen/office/FUSIONIFY-Spreadsheet.xlsx
+++ b/dokumen/office/FUSIONIFY-Spreadsheet.xlsx
@@ -1037,7 +1037,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>012/INV/FDS/X/2026</t>
+          <t>012/INV/FI/X/2026</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="D7" s="12" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
     </row>
     <row r="8">
@@ -1978,7 +1978,7 @@
         </is>
       </c>
       <c r="F10" s="39" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="G10" s="33" t="inlineStr">
         <is>

</xml_diff>